<commit_message>
Finally all the Save and Pend functionality is working. As far as I can tell anyway...
</commit_message>
<xml_diff>
--- a/documents/Outcomes upload.xlsx
+++ b/documents/Outcomes upload.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darryllrobinson/Documents/projects/ciab/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E843054A-5569-474F-A05C-0287F674EA0D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{215F8EBD-6D20-2F47-9C58-89820B99E862}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="28380" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="CaseOutcomes" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CaseOutcomes!$B$1:$R$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CaseOutcomes!$B$1:$Q$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="284">
   <si>
     <t>PTP</t>
   </si>
@@ -698,12 +698,6 @@
     <t>Resolution</t>
   </si>
   <si>
-    <t>NextVisitDate</t>
-  </si>
-  <si>
-    <t>NextVisitTime</t>
-  </si>
-  <si>
     <t>PhoneNumberCalled</t>
   </si>
   <si>
@@ -891,6 +885,9 @@
   </si>
   <si>
     <t>Retrace for contact info. (See Bureau report for Bukosini)</t>
+  </si>
+  <si>
+    <t>nextVisitDateTime</t>
   </si>
 </sst>
 </file>
@@ -962,7 +959,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1004,9 +1001,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1290,7 +1284,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0C429F0-77CD-4E06-B123-C56863115B7D}">
-  <dimension ref="A1:R596"/>
+  <dimension ref="A1:Q596"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="13" bestFit="1" customWidth="1"/>
@@ -1303,18 +1297,17 @@
     <col min="8" max="8" width="43.5" style="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.5" style="5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.6640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.5" style="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="26.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.5" style="5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.1640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.83203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="50.5" style="15" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.1640625" style="5"/>
+    <col min="11" max="11" width="17.83203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="26.5" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.5" style="5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.1640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="50.5" style="15" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.1640625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="3" customFormat="1" ht="14">
+    <row r="1" spans="1:17" s="3" customFormat="1" ht="14">
       <c r="A1" s="13" t="s">
         <v>208</v>
       </c>
@@ -1334,43 +1327,40 @@
         <v>188</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H1" s="20" t="s">
         <v>195</v>
       </c>
       <c r="I1" s="20" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J1" s="20" t="s">
         <v>219</v>
       </c>
-      <c r="K1" s="21" t="s">
-        <v>220</v>
+      <c r="K1" s="20" t="s">
+        <v>283</v>
       </c>
       <c r="L1" s="20" t="s">
-        <v>221</v>
+        <v>184</v>
       </c>
       <c r="M1" s="20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="N1" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O1" s="20" t="s">
-        <v>182</v>
+        <v>280</v>
       </c>
       <c r="P1" s="20" t="s">
-        <v>282</v>
-      </c>
-      <c r="Q1" s="20" t="s">
-        <v>283</v>
-      </c>
-      <c r="R1" s="18" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="28">
+        <v>281</v>
+      </c>
+      <c r="Q1" s="18" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="28">
       <c r="A2" s="13">
         <v>1</v>
       </c>
@@ -1378,7 +1368,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>213</v>
@@ -1399,24 +1389,21 @@
       <c r="J2" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="K2" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L2" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M2" s="8" t="s">
+      <c r="K2" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L2" s="8" t="s">
         <v>79</v>
       </c>
+      <c r="M2" s="8"/>
       <c r="N2" s="8"/>
       <c r="O2" s="8"/>
       <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="15" t="s">
+      <c r="Q2" s="15" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="14">
+    <row r="3" spans="1:17" ht="14">
       <c r="A3" s="13">
         <v>2</v>
       </c>
@@ -1424,7 +1411,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>213</v>
@@ -1445,20 +1432,17 @@
       <c r="J3" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="K3" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L3" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M3" s="5" t="s">
+      <c r="K3" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="R3" s="15" t="s">
+      <c r="Q3" s="15" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="14">
+    <row r="4" spans="1:17" ht="14">
       <c r="A4" s="13">
         <v>3</v>
       </c>
@@ -1466,7 +1450,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>213</v>
@@ -1484,20 +1468,17 @@
       <c r="J4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K4" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L4" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M4" s="5" t="s">
+      <c r="K4" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R4" s="15" t="s">
+      <c r="Q4" s="15" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="42">
+    <row r="5" spans="1:17" ht="42">
       <c r="A5" s="13">
         <v>4</v>
       </c>
@@ -1505,7 +1486,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>213</v>
@@ -1525,20 +1506,17 @@
       <c r="J5" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="K5" s="7">
-        <v>44040</v>
-      </c>
-      <c r="L5" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M5" s="5" t="s">
+      <c r="K5" s="12">
+        <v>44040.375</v>
+      </c>
+      <c r="L5" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="R5" s="15" t="s">
+      <c r="Q5" s="15" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="28">
+    <row r="6" spans="1:17" ht="28">
       <c r="A6" s="13">
         <v>4</v>
       </c>
@@ -1546,7 +1524,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>213</v>
@@ -1567,20 +1545,17 @@
       <c r="J6" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K6" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L6" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M6" s="5" t="s">
+      <c r="K6" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L6" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R6" s="15" t="s">
+      <c r="Q6" s="15" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="14">
+    <row r="7" spans="1:17" ht="14">
       <c r="A7" s="13">
         <v>5</v>
       </c>
@@ -1588,7 +1563,7 @@
         <v>7</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>213</v>
@@ -1609,20 +1584,17 @@
       <c r="J7" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="K7" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L7" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M7" s="5" t="s">
+      <c r="K7" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L7" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R7" s="15" t="s">
+      <c r="Q7" s="15" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="42">
+    <row r="8" spans="1:17" ht="42">
       <c r="A8" s="13">
         <v>6</v>
       </c>
@@ -1630,7 +1602,7 @@
         <v>8</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>213</v>
@@ -1653,20 +1625,17 @@
       <c r="J8" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="K8" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L8" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M8" s="5" t="s">
+      <c r="K8" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L8" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="R8" s="15" t="s">
+      <c r="Q8" s="15" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="14">
+    <row r="9" spans="1:17" ht="14">
       <c r="A9" s="13">
         <v>6</v>
       </c>
@@ -1674,7 +1643,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>213</v>
@@ -1689,20 +1658,17 @@
       <c r="J9" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="K9" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L9" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M9" s="5" t="s">
+      <c r="K9" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L9" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="R9" s="15" t="s">
+      <c r="Q9" s="15" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="14">
+    <row r="10" spans="1:17" ht="14">
       <c r="A10" s="13">
         <v>7</v>
       </c>
@@ -1710,7 +1676,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>213</v>
@@ -1731,20 +1697,17 @@
       <c r="J10" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="K10" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L10" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M10" s="5" t="s">
+      <c r="K10" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L10" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="R10" s="15" t="s">
+      <c r="Q10" s="15" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="42">
+    <row r="11" spans="1:17" ht="42">
       <c r="A11" s="13">
         <v>8</v>
       </c>
@@ -1752,7 +1715,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>213</v>
@@ -1773,20 +1736,17 @@
       <c r="J11" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="K11" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L11" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M11" s="5" t="s">
+      <c r="K11" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L11" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="R11" s="15" t="s">
+      <c r="Q11" s="15" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="14">
+    <row r="12" spans="1:17" ht="14">
       <c r="A12" s="13">
         <v>8</v>
       </c>
@@ -1794,7 +1754,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>213</v>
@@ -1813,20 +1773,17 @@
       <c r="J12" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="K12" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L12" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M12" s="5" t="s">
+      <c r="K12" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L12" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R12" s="15" t="s">
+      <c r="Q12" s="15" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="14">
+    <row r="13" spans="1:17" ht="14">
       <c r="A13" s="13">
         <v>9</v>
       </c>
@@ -1834,7 +1791,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>213</v>
@@ -1852,20 +1809,17 @@
       <c r="J13" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K13" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L13" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M13" s="5" t="s">
+      <c r="K13" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L13" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R13" s="15" t="s">
+      <c r="Q13" s="15" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="56">
+    <row r="14" spans="1:17" ht="56">
       <c r="A14" s="13">
         <v>10</v>
       </c>
@@ -1873,7 +1827,7 @@
         <v>12</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>213</v>
@@ -1894,20 +1848,17 @@
       <c r="J14" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="K14" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L14" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M14" s="5" t="s">
+      <c r="K14" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L14" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R14" s="15" t="s">
+      <c r="Q14" s="15" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="14">
+    <row r="15" spans="1:17" ht="14">
       <c r="A15" s="13">
         <v>12</v>
       </c>
@@ -1915,7 +1866,7 @@
         <v>13</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>213</v>
@@ -1933,20 +1884,17 @@
       <c r="J15" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K15" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L15" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M15" s="5" t="s">
+      <c r="K15" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L15" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R15" s="15" t="s">
+      <c r="Q15" s="15" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="42">
+    <row r="16" spans="1:17" ht="42">
       <c r="A16" s="13">
         <v>14</v>
       </c>
@@ -1954,7 +1902,7 @@
         <v>14</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>213</v>
@@ -1975,20 +1923,17 @@
       <c r="J16" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="K16" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L16" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M16" s="5" t="s">
+      <c r="K16" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L16" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="R16" s="15" t="s">
+      <c r="Q16" s="15" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="28">
+    <row r="17" spans="1:17" ht="28">
       <c r="A17" s="13">
         <v>15</v>
       </c>
@@ -1996,7 +1941,7 @@
         <v>15</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>213</v>
@@ -2016,20 +1961,17 @@
       <c r="J17" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K17" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L17" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M17" s="5" t="s">
+      <c r="K17" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L17" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R17" s="15" t="s">
+      <c r="Q17" s="15" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="14">
+    <row r="18" spans="1:17" ht="14">
       <c r="A18" s="13">
         <v>15</v>
       </c>
@@ -2037,7 +1979,7 @@
         <v>15</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>213</v>
@@ -2055,20 +1997,17 @@
       <c r="J18" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="K18" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L18" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M18" s="5" t="s">
+      <c r="K18" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L18" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R18" s="15" t="s">
+      <c r="Q18" s="15" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="14">
+    <row r="19" spans="1:17" ht="14">
       <c r="A19" s="13">
         <v>17</v>
       </c>
@@ -2076,7 +2015,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>213</v>
@@ -2094,20 +2033,17 @@
       <c r="J19" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K19" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L19" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M19" s="5" t="s">
+      <c r="K19" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L19" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R19" s="15" t="s">
+      <c r="Q19" s="15" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="14">
+    <row r="20" spans="1:17" ht="14">
       <c r="A20" s="13">
         <v>18</v>
       </c>
@@ -2115,7 +2051,7 @@
         <v>17</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>213</v>
@@ -2133,20 +2069,17 @@
       <c r="J20" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K20" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L20" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M20" s="5" t="s">
+      <c r="K20" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L20" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R20" s="15" t="s">
+      <c r="Q20" s="15" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="42">
+    <row r="21" spans="1:17" ht="42">
       <c r="A21" s="13">
         <v>18</v>
       </c>
@@ -2154,7 +2087,7 @@
         <v>17</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>213</v>
@@ -2174,20 +2107,17 @@
       <c r="J21" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="K21" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L21" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M21" s="5" t="s">
+      <c r="K21" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L21" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="R21" s="15" t="s">
+      <c r="Q21" s="15" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="14">
+    <row r="22" spans="1:17" ht="14">
       <c r="A22" s="13">
         <v>18</v>
       </c>
@@ -2195,7 +2125,7 @@
         <v>17</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>213</v>
@@ -2210,20 +2140,17 @@
       <c r="J22" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="K22" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L22" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M22" s="5" t="s">
+      <c r="K22" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L22" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="R22" s="15" t="s">
+      <c r="Q22" s="15" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="14">
+    <row r="23" spans="1:17" ht="14">
       <c r="A23" s="13">
         <v>19</v>
       </c>
@@ -2231,7 +2158,7 @@
         <v>18</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>213</v>
@@ -2249,20 +2176,17 @@
       <c r="J23" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K23" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L23" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M23" s="5" t="s">
+      <c r="K23" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L23" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R23" s="15" t="s">
+      <c r="Q23" s="15" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="14">
+    <row r="24" spans="1:17" ht="14">
       <c r="A24" s="13">
         <v>20</v>
       </c>
@@ -2270,7 +2194,7 @@
         <v>19</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>213</v>
@@ -2288,20 +2212,17 @@
       <c r="J24" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K24" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L24" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M24" s="5" t="s">
+      <c r="K24" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L24" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R24" s="15" t="s">
+      <c r="Q24" s="15" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="28">
+    <row r="25" spans="1:17" ht="28">
       <c r="A25" s="13">
         <v>21</v>
       </c>
@@ -2309,7 +2230,7 @@
         <v>20</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>213</v>
@@ -2332,20 +2253,17 @@
       <c r="J25" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="K25" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L25" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M25" s="5" t="s">
+      <c r="K25" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L25" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="R25" s="15" t="s">
+      <c r="Q25" s="15" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="28">
+    <row r="26" spans="1:17" ht="28">
       <c r="A26" s="13">
         <v>22</v>
       </c>
@@ -2353,7 +2271,7 @@
         <v>21</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>213</v>
@@ -2374,20 +2292,17 @@
       <c r="J26" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="K26" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L26" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M26" s="5" t="s">
+      <c r="K26" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L26" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="R26" s="15" t="s">
+      <c r="Q26" s="15" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="42">
+    <row r="27" spans="1:17" ht="42">
       <c r="A27" s="13">
         <v>23</v>
       </c>
@@ -2395,7 +2310,7 @@
         <v>22</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>213</v>
@@ -2415,20 +2330,17 @@
       <c r="J27" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="K27" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L27" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M27" s="5" t="s">
+      <c r="K27" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L27" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="R27" s="15" t="s">
+      <c r="Q27" s="15" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="14">
+    <row r="28" spans="1:17" ht="14">
       <c r="A28" s="13">
         <v>23</v>
       </c>
@@ -2436,7 +2348,7 @@
         <v>22</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>213</v>
@@ -2455,20 +2367,17 @@
       <c r="J28" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="K28" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L28" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M28" s="5" t="s">
+      <c r="K28" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L28" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R28" s="15" t="s">
+      <c r="Q28" s="15" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="14">
+    <row r="29" spans="1:17" ht="14">
       <c r="A29" s="13">
         <v>24</v>
       </c>
@@ -2476,7 +2385,7 @@
         <v>23</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>213</v>
@@ -2494,20 +2403,17 @@
       <c r="J29" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K29" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L29" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M29" s="5" t="s">
+      <c r="K29" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L29" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R29" s="15" t="s">
+      <c r="Q29" s="15" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="56">
+    <row r="30" spans="1:17" ht="56">
       <c r="A30" s="13">
         <v>25</v>
       </c>
@@ -2515,7 +2421,7 @@
         <v>24</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>213</v>
@@ -2536,20 +2442,17 @@
       <c r="J30" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="K30" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L30" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M30" s="5" t="s">
+      <c r="K30" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L30" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="R30" s="15" t="s">
+      <c r="Q30" s="15" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="28">
+    <row r="31" spans="1:17" ht="28">
       <c r="A31" s="13">
         <v>26</v>
       </c>
@@ -2557,7 +2460,7 @@
         <v>108</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>213</v>
@@ -2575,20 +2478,17 @@
       <c r="J31" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K31" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L31" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M31" s="5" t="s">
+      <c r="K31" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L31" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R31" s="15" t="s">
+      <c r="Q31" s="15" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="14">
+    <row r="32" spans="1:17" ht="14">
       <c r="A32" s="13">
         <v>27</v>
       </c>
@@ -2596,7 +2496,7 @@
         <v>25</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>213</v>
@@ -2619,20 +2519,17 @@
       <c r="J32" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="K32" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L32" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M32" s="5" t="s">
+      <c r="K32" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L32" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="R32" s="15" t="s">
+      <c r="Q32" s="15" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="14">
+    <row r="33" spans="1:17" ht="14">
       <c r="A33" s="13">
         <v>27</v>
       </c>
@@ -2640,7 +2537,7 @@
         <v>25</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>213</v>
@@ -2656,20 +2553,17 @@
       <c r="J33" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="K33" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L33" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M33" s="5" t="s">
+      <c r="K33" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L33" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R33" s="15" t="s">
+      <c r="Q33" s="15" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="56">
+    <row r="34" spans="1:17" ht="56">
       <c r="A34" s="13">
         <v>28</v>
       </c>
@@ -2677,7 +2571,7 @@
         <v>26</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>213</v>
@@ -2700,20 +2594,17 @@
       <c r="J34" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="K34" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L34" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M34" s="5" t="s">
+      <c r="K34" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L34" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="R34" s="15" t="s">
+      <c r="Q34" s="15" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="28">
+    <row r="35" spans="1:17" ht="28">
       <c r="A35" s="13">
         <v>28</v>
       </c>
@@ -2721,7 +2612,7 @@
         <v>26</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>213</v>
@@ -2737,20 +2628,17 @@
       <c r="J35" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="K35" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L35" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M35" s="5" t="s">
+      <c r="K35" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L35" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R35" s="15" t="s">
+      <c r="Q35" s="15" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="14">
+    <row r="36" spans="1:17" ht="14">
       <c r="A36" s="13">
         <v>29</v>
       </c>
@@ -2758,7 +2646,7 @@
         <v>27</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>213</v>
@@ -2776,20 +2664,17 @@
       <c r="J36" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K36" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L36" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M36" s="5" t="s">
+      <c r="K36" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L36" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R36" s="15" t="s">
+      <c r="Q36" s="15" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="14">
+    <row r="37" spans="1:17" ht="14">
       <c r="A37" s="13">
         <v>30</v>
       </c>
@@ -2797,7 +2682,7 @@
         <v>28</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>213</v>
@@ -2815,20 +2700,17 @@
       <c r="J37" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K37" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L37" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M37" s="5" t="s">
+      <c r="K37" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L37" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R37" s="15" t="s">
+      <c r="Q37" s="15" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="42">
+    <row r="38" spans="1:17" ht="42">
       <c r="A38" s="13">
         <v>31</v>
       </c>
@@ -2836,7 +2718,7 @@
         <v>29</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>213</v>
@@ -2857,20 +2739,17 @@
       <c r="J38" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="K38" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L38" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M38" s="5" t="s">
+      <c r="K38" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L38" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="R38" s="15" t="s">
+      <c r="Q38" s="15" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="28">
+    <row r="39" spans="1:17" ht="28">
       <c r="A39" s="13">
         <v>32</v>
       </c>
@@ -2878,7 +2757,7 @@
         <v>30</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>213</v>
@@ -2896,20 +2775,17 @@
       <c r="J39" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K39" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L39" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M39" s="5" t="s">
+      <c r="K39" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L39" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R39" s="15" t="s">
+      <c r="Q39" s="15" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="14">
+    <row r="40" spans="1:17" ht="14">
       <c r="A40" s="13">
         <v>33</v>
       </c>
@@ -2917,7 +2793,7 @@
         <v>31</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>213</v>
@@ -2937,20 +2813,17 @@
       <c r="J40" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="K40" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L40" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M40" s="5" t="s">
+      <c r="K40" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L40" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="R40" s="15" t="s">
+      <c r="Q40" s="15" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="42">
+    <row r="41" spans="1:17" ht="42">
       <c r="A41" s="13">
         <v>33</v>
       </c>
@@ -2958,7 +2831,7 @@
         <v>31</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>213</v>
@@ -2976,20 +2849,17 @@
       <c r="J41" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="K41" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L41" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M41" s="5" t="s">
+      <c r="K41" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L41" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R41" s="15" t="s">
+      <c r="Q41" s="15" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="14">
+    <row r="42" spans="1:17" ht="14">
       <c r="A42" s="13">
         <v>34</v>
       </c>
@@ -2997,7 +2867,7 @@
         <v>32</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>213</v>
@@ -3015,20 +2885,17 @@
       <c r="J42" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K42" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L42" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M42" s="5" t="s">
+      <c r="K42" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L42" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R42" s="15" t="s">
+      <c r="Q42" s="15" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="14">
+    <row r="43" spans="1:17" ht="14">
       <c r="A43" s="13">
         <v>34</v>
       </c>
@@ -3036,7 +2903,7 @@
         <v>32</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>213</v>
@@ -3054,20 +2921,17 @@
       <c r="J43" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K43" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L43" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M43" s="5" t="s">
+      <c r="K43" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L43" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R43" s="15" t="s">
+      <c r="Q43" s="15" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="14">
+    <row r="44" spans="1:17" ht="14">
       <c r="A44" s="13">
         <v>35</v>
       </c>
@@ -3075,7 +2939,7 @@
         <v>33</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>213</v>
@@ -3093,20 +2957,17 @@
       <c r="J44" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K44" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L44" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M44" s="5" t="s">
+      <c r="K44" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L44" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R44" s="15" t="s">
+      <c r="Q44" s="15" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="14">
+    <row r="45" spans="1:17" ht="14">
       <c r="A45" s="13">
         <v>37</v>
       </c>
@@ -3114,7 +2975,7 @@
         <v>35</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>213</v>
@@ -3132,20 +2993,17 @@
       <c r="J45" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K45" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L45" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M45" s="5" t="s">
+      <c r="K45" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L45" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R45" s="15" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="46" spans="1:18" ht="14">
+      <c r="Q45" s="15" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" ht="14">
       <c r="A46" s="13">
         <v>36</v>
       </c>
@@ -3153,7 +3011,7 @@
         <v>34</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>213</v>
@@ -3169,15 +3027,17 @@
       <c r="J46" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="L46" s="8"/>
-      <c r="M46" s="5" t="s">
+      <c r="K46" s="12">
+        <v>0</v>
+      </c>
+      <c r="L46" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="R46" s="15" t="s">
+      <c r="Q46" s="15" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="14">
+    <row r="47" spans="1:17" ht="14">
       <c r="A47" s="13">
         <v>38</v>
       </c>
@@ -3185,7 +3045,7 @@
         <v>36</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>213</v>
@@ -3208,20 +3068,17 @@
       <c r="J47" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="K47" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L47" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M47" s="5" t="s">
+      <c r="K47" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L47" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="R47" s="15" t="s">
+      <c r="Q47" s="15" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="14">
+    <row r="48" spans="1:17" ht="14">
       <c r="A48" s="13">
         <v>38</v>
       </c>
@@ -3229,7 +3086,7 @@
         <v>36</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>213</v>
@@ -3250,20 +3107,17 @@
       <c r="J48" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="K48" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L48" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M48" s="5" t="s">
+      <c r="K48" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L48" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R48" s="15" t="s">
+      <c r="Q48" s="15" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="28">
+    <row r="49" spans="1:17" ht="28">
       <c r="A49" s="13">
         <v>39</v>
       </c>
@@ -3271,7 +3125,7 @@
         <v>37</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>213</v>
@@ -3292,20 +3146,17 @@
       <c r="J49" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="K49" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L49" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M49" s="5" t="s">
+      <c r="K49" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L49" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="R49" s="15" t="s">
+      <c r="Q49" s="15" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="42">
+    <row r="50" spans="1:17" ht="42">
       <c r="A50" s="13">
         <v>40</v>
       </c>
@@ -3313,7 +3164,7 @@
         <v>38</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>213</v>
@@ -3334,20 +3185,17 @@
       <c r="J50" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="K50" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L50" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M50" s="5" t="s">
+      <c r="K50" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L50" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="R50" s="15" t="s">
+      <c r="Q50" s="15" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="14">
+    <row r="51" spans="1:17" ht="14">
       <c r="A51" s="13">
         <v>41</v>
       </c>
@@ -3355,7 +3203,7 @@
         <v>39</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>213</v>
@@ -3373,20 +3221,17 @@
       <c r="J51" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K51" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L51" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M51" s="5" t="s">
+      <c r="K51" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L51" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R51" s="15" t="s">
+      <c r="Q51" s="15" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="28">
+    <row r="52" spans="1:17" ht="28">
       <c r="A52" s="13">
         <v>42</v>
       </c>
@@ -3394,7 +3239,7 @@
         <v>40</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>213</v>
@@ -3411,20 +3256,17 @@
       <c r="J52" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="K52" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L52" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M52" s="5" t="s">
+      <c r="K52" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L52" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="R52" s="15" t="s">
+      <c r="Q52" s="15" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="28">
+    <row r="53" spans="1:17" ht="28">
       <c r="A53" s="13">
         <v>42</v>
       </c>
@@ -3432,7 +3274,7 @@
         <v>40</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>213</v>
@@ -3450,20 +3292,17 @@
       <c r="J53" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="K53" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L53" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M53" s="5" t="s">
+      <c r="K53" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L53" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="R53" s="15" t="s">
+      <c r="Q53" s="15" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="14">
+    <row r="54" spans="1:17" ht="14">
       <c r="A54" s="13">
         <v>43</v>
       </c>
@@ -3471,7 +3310,7 @@
         <v>41</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>213</v>
@@ -3489,20 +3328,17 @@
       <c r="J54" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K54" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L54" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M54" s="5" t="s">
+      <c r="K54" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L54" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R54" s="15" t="s">
+      <c r="Q54" s="15" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="28">
+    <row r="55" spans="1:17" ht="28">
       <c r="A55" s="13">
         <v>44</v>
       </c>
@@ -3510,7 +3346,7 @@
         <v>42</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>213</v>
@@ -3530,20 +3366,17 @@
       <c r="J55" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="K55" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L55" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M55" s="5" t="s">
+      <c r="K55" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L55" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="R55" s="15" t="s">
+      <c r="Q55" s="15" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="14">
+    <row r="56" spans="1:17" ht="14">
       <c r="A56" s="13">
         <v>44</v>
       </c>
@@ -3551,7 +3384,7 @@
         <v>42</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>213</v>
@@ -3569,20 +3402,17 @@
       <c r="J56" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="K56" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L56" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M56" s="5" t="s">
+      <c r="K56" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L56" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R56" s="15" t="s">
+      <c r="Q56" s="15" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="14">
+    <row r="57" spans="1:17" ht="14">
       <c r="A57" s="13">
         <v>45</v>
       </c>
@@ -3590,7 +3420,7 @@
         <v>43</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>213</v>
@@ -3611,20 +3441,17 @@
       <c r="J57" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="K57" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L57" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M57" s="5" t="s">
+      <c r="K57" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L57" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R57" s="15" t="s">
+      <c r="Q57" s="15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="42">
+    <row r="58" spans="1:17" ht="42">
       <c r="A58" s="13">
         <v>46</v>
       </c>
@@ -3632,7 +3459,7 @@
         <v>44</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>213</v>
@@ -3655,20 +3482,17 @@
       <c r="J58" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="K58" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L58" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M58" s="5" t="s">
+      <c r="K58" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L58" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="R58" s="15" t="s">
+      <c r="Q58" s="15" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="28">
+    <row r="59" spans="1:17" ht="28">
       <c r="A59" s="13">
         <v>47</v>
       </c>
@@ -3676,7 +3500,7 @@
         <v>45</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>213</v>
@@ -3697,20 +3521,17 @@
       <c r="J59" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="K59" s="7">
-        <v>44063</v>
-      </c>
-      <c r="L59" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M59" s="5" t="s">
+      <c r="K59" s="12">
+        <v>44063.375</v>
+      </c>
+      <c r="L59" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R59" s="15" t="s">
+      <c r="Q59" s="15" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="42">
+    <row r="60" spans="1:17" ht="42">
       <c r="A60" s="13">
         <v>48</v>
       </c>
@@ -3718,7 +3539,7 @@
         <v>46</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D60" s="1" t="s">
         <v>213</v>
@@ -3739,20 +3560,17 @@
       <c r="J60" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="K60" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L60" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M60" s="5" t="s">
+      <c r="K60" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L60" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="R60" s="15" t="s">
+      <c r="Q60" s="15" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="14">
+    <row r="61" spans="1:17" ht="14">
       <c r="A61" s="13">
         <v>49</v>
       </c>
@@ -3760,7 +3578,7 @@
         <v>47</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>213</v>
@@ -3778,20 +3596,17 @@
       <c r="J61" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K61" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L61" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M61" s="5" t="s">
+      <c r="K61" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L61" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R61" s="15" t="s">
+      <c r="Q61" s="15" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="28">
+    <row r="62" spans="1:17" ht="28">
       <c r="A62" s="13">
         <v>50</v>
       </c>
@@ -3799,7 +3614,7 @@
         <v>48</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>213</v>
@@ -3817,121 +3632,118 @@
       <c r="J62" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="K62" s="7">
-        <v>44048</v>
-      </c>
-      <c r="L62" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="M62" s="5" t="s">
+      <c r="K62" s="12">
+        <v>44048.375</v>
+      </c>
+      <c r="L62" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="R62" s="15" t="s">
+      <c r="Q62" s="15" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="63" spans="1:18">
+    <row r="63" spans="1:17">
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
       <c r="G63" s="2"/>
       <c r="H63" s="7"/>
-      <c r="L63" s="8"/>
-    </row>
-    <row r="64" spans="1:18">
+      <c r="K63" s="8"/>
+    </row>
+    <row r="64" spans="1:17">
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
       <c r="H64" s="7"/>
     </row>
-    <row r="65" spans="2:12">
+    <row r="65" spans="2:11">
       <c r="B65" s="1"/>
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
       <c r="G65" s="2"/>
       <c r="H65" s="7"/>
-      <c r="L65" s="8"/>
-    </row>
-    <row r="66" spans="2:12">
+      <c r="K65" s="8"/>
+    </row>
+    <row r="66" spans="2:11">
       <c r="D66" s="1"/>
       <c r="E66" s="1"/>
       <c r="F66" s="1"/>
       <c r="G66" s="2"/>
       <c r="H66" s="7"/>
-      <c r="L66" s="8"/>
-    </row>
-    <row r="67" spans="2:12">
+      <c r="K66" s="8"/>
+    </row>
+    <row r="67" spans="2:11">
       <c r="B67" s="1"/>
       <c r="D67" s="1"/>
       <c r="E67" s="1"/>
       <c r="F67" s="1"/>
       <c r="G67" s="2"/>
       <c r="H67" s="7"/>
-      <c r="L67" s="8"/>
-    </row>
-    <row r="68" spans="2:12">
+      <c r="K67" s="8"/>
+    </row>
+    <row r="68" spans="2:11">
       <c r="H68" s="7"/>
     </row>
-    <row r="69" spans="2:12">
+    <row r="69" spans="2:11">
       <c r="H69" s="7"/>
     </row>
-    <row r="70" spans="2:12">
+    <row r="70" spans="2:11">
       <c r="H70" s="7"/>
     </row>
-    <row r="71" spans="2:12">
+    <row r="71" spans="2:11">
       <c r="D71" s="1"/>
       <c r="E71" s="1"/>
       <c r="F71" s="1"/>
       <c r="H71" s="7"/>
     </row>
-    <row r="72" spans="2:12">
+    <row r="72" spans="2:11">
       <c r="D72" s="1"/>
       <c r="E72" s="1"/>
       <c r="F72" s="1"/>
       <c r="H72" s="7"/>
     </row>
-    <row r="73" spans="2:12">
+    <row r="73" spans="2:11">
       <c r="D73" s="1"/>
       <c r="E73" s="1"/>
       <c r="F73" s="1"/>
       <c r="G73" s="2"/>
       <c r="H73" s="10"/>
     </row>
-    <row r="74" spans="2:12">
+    <row r="74" spans="2:11">
       <c r="D74" s="1"/>
       <c r="E74" s="1"/>
       <c r="F74" s="1"/>
       <c r="H74" s="7"/>
     </row>
-    <row r="75" spans="2:12">
+    <row r="75" spans="2:11">
       <c r="D75" s="1"/>
       <c r="E75" s="1"/>
       <c r="F75" s="1"/>
       <c r="H75" s="7"/>
     </row>
-    <row r="76" spans="2:12">
+    <row r="76" spans="2:11">
       <c r="D76" s="1"/>
       <c r="E76" s="1"/>
       <c r="F76" s="1"/>
       <c r="H76" s="7"/>
     </row>
-    <row r="77" spans="2:12">
+    <row r="77" spans="2:11">
       <c r="D77" s="1"/>
       <c r="E77" s="1"/>
       <c r="F77" s="1"/>
       <c r="H77" s="7"/>
     </row>
-    <row r="78" spans="2:12">
+    <row r="78" spans="2:11">
       <c r="D78" s="1"/>
       <c r="E78" s="1"/>
       <c r="F78" s="1"/>
       <c r="H78" s="7"/>
     </row>
-    <row r="79" spans="2:12">
+    <row r="79" spans="2:11">
       <c r="H79" s="7"/>
     </row>
-    <row r="80" spans="2:12">
+    <row r="80" spans="2:11">
       <c r="H80" s="7"/>
     </row>
     <row r="81" spans="8:8">
@@ -5038,851 +4850,851 @@
     <row r="448" spans="8:8">
       <c r="H448" s="7"/>
     </row>
-    <row r="449" spans="1:18">
+    <row r="449" spans="1:17">
       <c r="H449" s="7"/>
     </row>
-    <row r="457" spans="1:18" s="7" customFormat="1">
+    <row r="457" spans="1:17" s="7" customFormat="1">
       <c r="A457" s="13"/>
       <c r="C457" s="12"/>
       <c r="G457" s="6"/>
-      <c r="R457" s="16"/>
-    </row>
-    <row r="458" spans="1:18" s="7" customFormat="1">
+      <c r="Q457" s="16"/>
+    </row>
+    <row r="458" spans="1:17" s="7" customFormat="1">
       <c r="A458" s="13"/>
       <c r="C458" s="12"/>
       <c r="G458" s="6"/>
-      <c r="R458" s="16"/>
-    </row>
-    <row r="459" spans="1:18" s="7" customFormat="1">
+      <c r="Q458" s="16"/>
+    </row>
+    <row r="459" spans="1:17" s="7" customFormat="1">
       <c r="A459" s="13"/>
       <c r="C459" s="12"/>
       <c r="G459" s="6"/>
-      <c r="R459" s="16"/>
-    </row>
-    <row r="460" spans="1:18" s="7" customFormat="1">
+      <c r="Q459" s="16"/>
+    </row>
+    <row r="460" spans="1:17" s="7" customFormat="1">
       <c r="A460" s="13"/>
       <c r="C460" s="12"/>
       <c r="G460" s="6"/>
-      <c r="R460" s="16"/>
-    </row>
-    <row r="461" spans="1:18" s="7" customFormat="1">
+      <c r="Q460" s="16"/>
+    </row>
+    <row r="461" spans="1:17" s="7" customFormat="1">
       <c r="A461" s="13"/>
       <c r="C461" s="12"/>
       <c r="G461" s="6"/>
-      <c r="R461" s="16"/>
-    </row>
-    <row r="462" spans="1:18" s="7" customFormat="1">
+      <c r="Q461" s="16"/>
+    </row>
+    <row r="462" spans="1:17" s="7" customFormat="1">
       <c r="A462" s="13"/>
       <c r="C462" s="12"/>
       <c r="G462" s="6"/>
-      <c r="R462" s="16"/>
-    </row>
-    <row r="463" spans="1:18" s="7" customFormat="1">
+      <c r="Q462" s="16"/>
+    </row>
+    <row r="463" spans="1:17" s="7" customFormat="1">
       <c r="A463" s="13"/>
       <c r="C463" s="12"/>
       <c r="G463" s="6"/>
-      <c r="R463" s="16"/>
-    </row>
-    <row r="464" spans="1:18" s="7" customFormat="1">
+      <c r="Q463" s="16"/>
+    </row>
+    <row r="464" spans="1:17" s="7" customFormat="1">
       <c r="A464" s="13"/>
       <c r="C464" s="12"/>
       <c r="G464" s="6"/>
-      <c r="R464" s="16"/>
-    </row>
-    <row r="465" spans="1:18" s="7" customFormat="1">
+      <c r="Q464" s="16"/>
+    </row>
+    <row r="465" spans="1:17" s="7" customFormat="1">
       <c r="A465" s="13"/>
       <c r="C465" s="12"/>
       <c r="G465" s="6"/>
-      <c r="R465" s="16"/>
-    </row>
-    <row r="466" spans="1:18" s="7" customFormat="1">
+      <c r="Q465" s="16"/>
+    </row>
+    <row r="466" spans="1:17" s="7" customFormat="1">
       <c r="A466" s="13"/>
       <c r="C466" s="12"/>
       <c r="G466" s="6"/>
-      <c r="R466" s="16"/>
-    </row>
-    <row r="467" spans="1:18" s="7" customFormat="1">
+      <c r="Q466" s="16"/>
+    </row>
+    <row r="467" spans="1:17" s="7" customFormat="1">
       <c r="A467" s="13"/>
       <c r="C467" s="12"/>
       <c r="G467" s="6"/>
-      <c r="R467" s="16"/>
-    </row>
-    <row r="468" spans="1:18" s="7" customFormat="1">
+      <c r="Q467" s="16"/>
+    </row>
+    <row r="468" spans="1:17" s="7" customFormat="1">
       <c r="A468" s="13"/>
       <c r="C468" s="12"/>
       <c r="G468" s="6"/>
-      <c r="R468" s="16"/>
-    </row>
-    <row r="469" spans="1:18" s="7" customFormat="1">
+      <c r="Q468" s="16"/>
+    </row>
+    <row r="469" spans="1:17" s="7" customFormat="1">
       <c r="A469" s="13"/>
       <c r="C469" s="12"/>
       <c r="G469" s="6"/>
-      <c r="R469" s="16"/>
-    </row>
-    <row r="470" spans="1:18" s="7" customFormat="1">
+      <c r="Q469" s="16"/>
+    </row>
+    <row r="470" spans="1:17" s="7" customFormat="1">
       <c r="A470" s="13"/>
       <c r="C470" s="12"/>
       <c r="G470" s="6"/>
-      <c r="R470" s="16"/>
-    </row>
-    <row r="471" spans="1:18" s="7" customFormat="1">
+      <c r="Q470" s="16"/>
+    </row>
+    <row r="471" spans="1:17" s="7" customFormat="1">
       <c r="A471" s="13"/>
       <c r="C471" s="12"/>
       <c r="G471" s="6"/>
-      <c r="R471" s="16"/>
-    </row>
-    <row r="472" spans="1:18" s="7" customFormat="1">
+      <c r="Q471" s="16"/>
+    </row>
+    <row r="472" spans="1:17" s="7" customFormat="1">
       <c r="A472" s="13"/>
       <c r="C472" s="12"/>
       <c r="G472" s="6"/>
-      <c r="R472" s="16"/>
-    </row>
-    <row r="473" spans="1:18" s="7" customFormat="1">
+      <c r="Q472" s="16"/>
+    </row>
+    <row r="473" spans="1:17" s="7" customFormat="1">
       <c r="A473" s="13"/>
       <c r="C473" s="12"/>
       <c r="G473" s="6"/>
-      <c r="R473" s="16"/>
-    </row>
-    <row r="474" spans="1:18" s="7" customFormat="1">
+      <c r="Q473" s="16"/>
+    </row>
+    <row r="474" spans="1:17" s="7" customFormat="1">
       <c r="A474" s="13"/>
       <c r="C474" s="12"/>
       <c r="G474" s="6"/>
-      <c r="R474" s="16"/>
-    </row>
-    <row r="475" spans="1:18" s="7" customFormat="1">
+      <c r="Q474" s="16"/>
+    </row>
+    <row r="475" spans="1:17" s="7" customFormat="1">
       <c r="A475" s="13"/>
       <c r="C475" s="12"/>
       <c r="G475" s="6"/>
-      <c r="R475" s="16"/>
-    </row>
-    <row r="476" spans="1:18" s="7" customFormat="1">
+      <c r="Q475" s="16"/>
+    </row>
+    <row r="476" spans="1:17" s="7" customFormat="1">
       <c r="A476" s="13"/>
       <c r="C476" s="12"/>
       <c r="G476" s="6"/>
-      <c r="R476" s="16"/>
-    </row>
-    <row r="477" spans="1:18" s="7" customFormat="1">
+      <c r="Q476" s="16"/>
+    </row>
+    <row r="477" spans="1:17" s="7" customFormat="1">
       <c r="A477" s="13"/>
       <c r="C477" s="12"/>
       <c r="G477" s="6"/>
-      <c r="R477" s="16"/>
-    </row>
-    <row r="478" spans="1:18" s="7" customFormat="1">
+      <c r="Q477" s="16"/>
+    </row>
+    <row r="478" spans="1:17" s="7" customFormat="1">
       <c r="A478" s="13"/>
       <c r="C478" s="12"/>
       <c r="G478" s="6"/>
-      <c r="R478" s="16"/>
-    </row>
-    <row r="479" spans="1:18" s="7" customFormat="1">
+      <c r="Q478" s="16"/>
+    </row>
+    <row r="479" spans="1:17" s="7" customFormat="1">
       <c r="A479" s="13"/>
       <c r="C479" s="12"/>
       <c r="G479" s="6"/>
-      <c r="R479" s="16"/>
-    </row>
-    <row r="480" spans="1:18" s="7" customFormat="1">
+      <c r="Q479" s="16"/>
+    </row>
+    <row r="480" spans="1:17" s="7" customFormat="1">
       <c r="A480" s="13"/>
       <c r="C480" s="12"/>
       <c r="G480" s="6"/>
-      <c r="R480" s="16"/>
-    </row>
-    <row r="481" spans="1:18" s="7" customFormat="1">
+      <c r="Q480" s="16"/>
+    </row>
+    <row r="481" spans="1:17" s="7" customFormat="1">
       <c r="A481" s="13"/>
       <c r="C481" s="12"/>
       <c r="G481" s="6"/>
-      <c r="R481" s="16"/>
-    </row>
-    <row r="482" spans="1:18" s="7" customFormat="1">
+      <c r="Q481" s="16"/>
+    </row>
+    <row r="482" spans="1:17" s="7" customFormat="1">
       <c r="A482" s="13"/>
       <c r="C482" s="12"/>
       <c r="G482" s="6"/>
-      <c r="R482" s="16"/>
-    </row>
-    <row r="483" spans="1:18" s="7" customFormat="1">
+      <c r="Q482" s="16"/>
+    </row>
+    <row r="483" spans="1:17" s="7" customFormat="1">
       <c r="A483" s="13"/>
       <c r="C483" s="12"/>
       <c r="G483" s="6"/>
-      <c r="R483" s="16"/>
-    </row>
-    <row r="484" spans="1:18" s="7" customFormat="1">
+      <c r="Q483" s="16"/>
+    </row>
+    <row r="484" spans="1:17" s="7" customFormat="1">
       <c r="A484" s="13"/>
       <c r="C484" s="12"/>
       <c r="G484" s="6"/>
-      <c r="R484" s="16"/>
-    </row>
-    <row r="485" spans="1:18" s="7" customFormat="1">
+      <c r="Q484" s="16"/>
+    </row>
+    <row r="485" spans="1:17" s="7" customFormat="1">
       <c r="A485" s="13"/>
       <c r="C485" s="12"/>
       <c r="G485" s="6"/>
-      <c r="R485" s="16"/>
-    </row>
-    <row r="486" spans="1:18" s="7" customFormat="1">
+      <c r="Q485" s="16"/>
+    </row>
+    <row r="486" spans="1:17" s="7" customFormat="1">
       <c r="A486" s="13"/>
       <c r="C486" s="12"/>
       <c r="G486" s="6"/>
-      <c r="R486" s="16"/>
-    </row>
-    <row r="487" spans="1:18" s="7" customFormat="1">
+      <c r="Q486" s="16"/>
+    </row>
+    <row r="487" spans="1:17" s="7" customFormat="1">
       <c r="A487" s="13"/>
       <c r="C487" s="12"/>
       <c r="G487" s="6"/>
-      <c r="R487" s="16"/>
-    </row>
-    <row r="488" spans="1:18" s="7" customFormat="1">
+      <c r="Q487" s="16"/>
+    </row>
+    <row r="488" spans="1:17" s="7" customFormat="1">
       <c r="A488" s="13"/>
       <c r="C488" s="12"/>
       <c r="G488" s="6"/>
-      <c r="R488" s="16"/>
-    </row>
-    <row r="489" spans="1:18" s="7" customFormat="1">
+      <c r="Q488" s="16"/>
+    </row>
+    <row r="489" spans="1:17" s="7" customFormat="1">
       <c r="A489" s="13"/>
       <c r="C489" s="12"/>
       <c r="G489" s="6"/>
-      <c r="R489" s="16"/>
-    </row>
-    <row r="490" spans="1:18" s="7" customFormat="1">
+      <c r="Q489" s="16"/>
+    </row>
+    <row r="490" spans="1:17" s="7" customFormat="1">
       <c r="A490" s="13"/>
       <c r="C490" s="12"/>
       <c r="G490" s="6"/>
-      <c r="R490" s="16"/>
-    </row>
-    <row r="491" spans="1:18" s="7" customFormat="1">
+      <c r="Q490" s="16"/>
+    </row>
+    <row r="491" spans="1:17" s="7" customFormat="1">
       <c r="A491" s="13"/>
       <c r="C491" s="12"/>
       <c r="G491" s="6"/>
-      <c r="R491" s="16"/>
-    </row>
-    <row r="492" spans="1:18" s="7" customFormat="1">
+      <c r="Q491" s="16"/>
+    </row>
+    <row r="492" spans="1:17" s="7" customFormat="1">
       <c r="A492" s="13"/>
       <c r="C492" s="12"/>
       <c r="G492" s="6"/>
-      <c r="R492" s="16"/>
-    </row>
-    <row r="493" spans="1:18" s="7" customFormat="1">
+      <c r="Q492" s="16"/>
+    </row>
+    <row r="493" spans="1:17" s="7" customFormat="1">
       <c r="A493" s="13"/>
       <c r="C493" s="12"/>
       <c r="G493" s="6"/>
-      <c r="R493" s="16"/>
-    </row>
-    <row r="494" spans="1:18" s="7" customFormat="1">
+      <c r="Q493" s="16"/>
+    </row>
+    <row r="494" spans="1:17" s="7" customFormat="1">
       <c r="A494" s="13"/>
       <c r="C494" s="12"/>
       <c r="G494" s="6"/>
-      <c r="R494" s="16"/>
-    </row>
-    <row r="495" spans="1:18" s="7" customFormat="1">
+      <c r="Q494" s="16"/>
+    </row>
+    <row r="495" spans="1:17" s="7" customFormat="1">
       <c r="A495" s="13"/>
       <c r="C495" s="12"/>
       <c r="G495" s="6"/>
-      <c r="R495" s="16"/>
-    </row>
-    <row r="496" spans="1:18" s="7" customFormat="1">
+      <c r="Q495" s="16"/>
+    </row>
+    <row r="496" spans="1:17" s="7" customFormat="1">
       <c r="A496" s="13"/>
       <c r="C496" s="12"/>
       <c r="G496" s="6"/>
-      <c r="R496" s="16"/>
-    </row>
-    <row r="497" spans="1:18" s="7" customFormat="1">
+      <c r="Q496" s="16"/>
+    </row>
+    <row r="497" spans="1:17" s="7" customFormat="1">
       <c r="A497" s="13"/>
       <c r="C497" s="12"/>
       <c r="G497" s="6"/>
-      <c r="R497" s="16"/>
-    </row>
-    <row r="498" spans="1:18" s="7" customFormat="1">
+      <c r="Q497" s="16"/>
+    </row>
+    <row r="498" spans="1:17" s="7" customFormat="1">
       <c r="A498" s="13"/>
       <c r="C498" s="12"/>
       <c r="G498" s="6"/>
-      <c r="R498" s="16"/>
-    </row>
-    <row r="499" spans="1:18" s="7" customFormat="1">
+      <c r="Q498" s="16"/>
+    </row>
+    <row r="499" spans="1:17" s="7" customFormat="1">
       <c r="A499" s="13"/>
       <c r="C499" s="12"/>
       <c r="G499" s="6"/>
-      <c r="R499" s="16"/>
-    </row>
-    <row r="500" spans="1:18" s="7" customFormat="1">
+      <c r="Q499" s="16"/>
+    </row>
+    <row r="500" spans="1:17" s="7" customFormat="1">
       <c r="A500" s="13"/>
       <c r="C500" s="12"/>
       <c r="G500" s="6"/>
-      <c r="R500" s="16"/>
-    </row>
-    <row r="501" spans="1:18" s="7" customFormat="1">
+      <c r="Q500" s="16"/>
+    </row>
+    <row r="501" spans="1:17" s="7" customFormat="1">
       <c r="A501" s="13"/>
       <c r="C501" s="12"/>
       <c r="G501" s="6"/>
-      <c r="R501" s="16"/>
-    </row>
-    <row r="502" spans="1:18" s="7" customFormat="1">
+      <c r="Q501" s="16"/>
+    </row>
+    <row r="502" spans="1:17" s="7" customFormat="1">
       <c r="A502" s="13"/>
       <c r="C502" s="12"/>
       <c r="G502" s="6"/>
-      <c r="R502" s="16"/>
-    </row>
-    <row r="503" spans="1:18" s="7" customFormat="1">
+      <c r="Q502" s="16"/>
+    </row>
+    <row r="503" spans="1:17" s="7" customFormat="1">
       <c r="A503" s="13"/>
       <c r="C503" s="12"/>
       <c r="G503" s="6"/>
-      <c r="R503" s="16"/>
-    </row>
-    <row r="504" spans="1:18" s="7" customFormat="1">
+      <c r="Q503" s="16"/>
+    </row>
+    <row r="504" spans="1:17" s="7" customFormat="1">
       <c r="A504" s="13"/>
       <c r="C504" s="12"/>
       <c r="G504" s="6"/>
-      <c r="R504" s="16"/>
-    </row>
-    <row r="505" spans="1:18" s="7" customFormat="1">
+      <c r="Q504" s="16"/>
+    </row>
+    <row r="505" spans="1:17" s="7" customFormat="1">
       <c r="A505" s="13"/>
       <c r="C505" s="12"/>
       <c r="G505" s="6"/>
-      <c r="R505" s="16"/>
-    </row>
-    <row r="506" spans="1:18" s="7" customFormat="1">
+      <c r="Q505" s="16"/>
+    </row>
+    <row r="506" spans="1:17" s="7" customFormat="1">
       <c r="A506" s="13"/>
       <c r="C506" s="12"/>
       <c r="G506" s="6"/>
-      <c r="R506" s="16"/>
-    </row>
-    <row r="507" spans="1:18" s="7" customFormat="1">
+      <c r="Q506" s="16"/>
+    </row>
+    <row r="507" spans="1:17" s="7" customFormat="1">
       <c r="A507" s="13"/>
       <c r="C507" s="12"/>
       <c r="G507" s="6"/>
-      <c r="R507" s="16"/>
-    </row>
-    <row r="508" spans="1:18" s="7" customFormat="1">
+      <c r="Q507" s="16"/>
+    </row>
+    <row r="508" spans="1:17" s="7" customFormat="1">
       <c r="A508" s="13"/>
       <c r="C508" s="12"/>
       <c r="G508" s="6"/>
-      <c r="R508" s="16"/>
-    </row>
-    <row r="509" spans="1:18" s="7" customFormat="1">
+      <c r="Q508" s="16"/>
+    </row>
+    <row r="509" spans="1:17" s="7" customFormat="1">
       <c r="A509" s="13"/>
       <c r="C509" s="12"/>
       <c r="G509" s="6"/>
-      <c r="R509" s="16"/>
-    </row>
-    <row r="510" spans="1:18" s="7" customFormat="1">
+      <c r="Q509" s="16"/>
+    </row>
+    <row r="510" spans="1:17" s="7" customFormat="1">
       <c r="A510" s="13"/>
       <c r="C510" s="12"/>
       <c r="G510" s="6"/>
-      <c r="R510" s="16"/>
-    </row>
-    <row r="511" spans="1:18" s="7" customFormat="1">
+      <c r="Q510" s="16"/>
+    </row>
+    <row r="511" spans="1:17" s="7" customFormat="1">
       <c r="A511" s="13"/>
       <c r="C511" s="12"/>
       <c r="G511" s="6"/>
-      <c r="R511" s="16"/>
-    </row>
-    <row r="512" spans="1:18" s="7" customFormat="1">
+      <c r="Q511" s="16"/>
+    </row>
+    <row r="512" spans="1:17" s="7" customFormat="1">
       <c r="A512" s="13"/>
       <c r="C512" s="12"/>
       <c r="G512" s="6"/>
-      <c r="R512" s="16"/>
-    </row>
-    <row r="513" spans="1:18" s="7" customFormat="1">
+      <c r="Q512" s="16"/>
+    </row>
+    <row r="513" spans="1:17" s="7" customFormat="1">
       <c r="A513" s="13"/>
       <c r="C513" s="12"/>
       <c r="G513" s="6"/>
-      <c r="R513" s="16"/>
-    </row>
-    <row r="514" spans="1:18" s="7" customFormat="1">
+      <c r="Q513" s="16"/>
+    </row>
+    <row r="514" spans="1:17" s="7" customFormat="1">
       <c r="A514" s="13"/>
       <c r="C514" s="12"/>
       <c r="G514" s="6"/>
-      <c r="R514" s="16"/>
-    </row>
-    <row r="515" spans="1:18" s="7" customFormat="1">
+      <c r="Q514" s="16"/>
+    </row>
+    <row r="515" spans="1:17" s="7" customFormat="1">
       <c r="A515" s="13"/>
       <c r="C515" s="12"/>
       <c r="G515" s="6"/>
-      <c r="R515" s="16"/>
-    </row>
-    <row r="516" spans="1:18" s="7" customFormat="1">
+      <c r="Q515" s="16"/>
+    </row>
+    <row r="516" spans="1:17" s="7" customFormat="1">
       <c r="A516" s="13"/>
       <c r="C516" s="12"/>
       <c r="G516" s="6"/>
-      <c r="R516" s="16"/>
-    </row>
-    <row r="517" spans="1:18" s="7" customFormat="1">
+      <c r="Q516" s="16"/>
+    </row>
+    <row r="517" spans="1:17" s="7" customFormat="1">
       <c r="A517" s="13"/>
       <c r="C517" s="12"/>
       <c r="G517" s="6"/>
-      <c r="R517" s="16"/>
-    </row>
-    <row r="518" spans="1:18" s="7" customFormat="1">
+      <c r="Q517" s="16"/>
+    </row>
+    <row r="518" spans="1:17" s="7" customFormat="1">
       <c r="A518" s="13"/>
       <c r="C518" s="12"/>
       <c r="G518" s="6"/>
-      <c r="R518" s="16"/>
-    </row>
-    <row r="519" spans="1:18" s="7" customFormat="1">
+      <c r="Q518" s="16"/>
+    </row>
+    <row r="519" spans="1:17" s="7" customFormat="1">
       <c r="A519" s="13"/>
       <c r="C519" s="12"/>
       <c r="G519" s="6"/>
-      <c r="R519" s="16"/>
-    </row>
-    <row r="520" spans="1:18" s="7" customFormat="1">
+      <c r="Q519" s="16"/>
+    </row>
+    <row r="520" spans="1:17" s="7" customFormat="1">
       <c r="A520" s="13"/>
       <c r="C520" s="12"/>
       <c r="G520" s="6"/>
-      <c r="R520" s="16"/>
-    </row>
-    <row r="521" spans="1:18" s="7" customFormat="1">
+      <c r="Q520" s="16"/>
+    </row>
+    <row r="521" spans="1:17" s="7" customFormat="1">
       <c r="A521" s="13"/>
       <c r="C521" s="12"/>
       <c r="G521" s="6"/>
-      <c r="R521" s="16"/>
-    </row>
-    <row r="522" spans="1:18" s="7" customFormat="1">
+      <c r="Q521" s="16"/>
+    </row>
+    <row r="522" spans="1:17" s="7" customFormat="1">
       <c r="A522" s="13"/>
       <c r="C522" s="12"/>
       <c r="G522" s="6"/>
-      <c r="R522" s="16"/>
-    </row>
-    <row r="523" spans="1:18" s="7" customFormat="1">
+      <c r="Q522" s="16"/>
+    </row>
+    <row r="523" spans="1:17" s="7" customFormat="1">
       <c r="A523" s="13"/>
       <c r="C523" s="12"/>
       <c r="G523" s="6"/>
-      <c r="R523" s="16"/>
-    </row>
-    <row r="524" spans="1:18" s="7" customFormat="1">
+      <c r="Q523" s="16"/>
+    </row>
+    <row r="524" spans="1:17" s="7" customFormat="1">
       <c r="A524" s="13"/>
       <c r="C524" s="12"/>
       <c r="G524" s="6"/>
-      <c r="R524" s="16"/>
-    </row>
-    <row r="525" spans="1:18" s="7" customFormat="1">
+      <c r="Q524" s="16"/>
+    </row>
+    <row r="525" spans="1:17" s="7" customFormat="1">
       <c r="A525" s="13"/>
       <c r="C525" s="12"/>
       <c r="G525" s="6"/>
-      <c r="R525" s="16"/>
-    </row>
-    <row r="526" spans="1:18" s="7" customFormat="1">
+      <c r="Q525" s="16"/>
+    </row>
+    <row r="526" spans="1:17" s="7" customFormat="1">
       <c r="A526" s="13"/>
       <c r="C526" s="12"/>
       <c r="G526" s="6"/>
-      <c r="R526" s="16"/>
-    </row>
-    <row r="527" spans="1:18" s="7" customFormat="1">
+      <c r="Q526" s="16"/>
+    </row>
+    <row r="527" spans="1:17" s="7" customFormat="1">
       <c r="A527" s="13"/>
       <c r="C527" s="12"/>
       <c r="G527" s="6"/>
-      <c r="R527" s="16"/>
-    </row>
-    <row r="528" spans="1:18" s="7" customFormat="1">
+      <c r="Q527" s="16"/>
+    </row>
+    <row r="528" spans="1:17" s="7" customFormat="1">
       <c r="A528" s="13"/>
       <c r="C528" s="12"/>
       <c r="G528" s="6"/>
-      <c r="R528" s="16"/>
-    </row>
-    <row r="529" spans="1:18" s="7" customFormat="1">
+      <c r="Q528" s="16"/>
+    </row>
+    <row r="529" spans="1:17" s="7" customFormat="1">
       <c r="A529" s="13"/>
       <c r="C529" s="12"/>
       <c r="G529" s="6"/>
-      <c r="R529" s="16"/>
-    </row>
-    <row r="530" spans="1:18" s="7" customFormat="1">
+      <c r="Q529" s="16"/>
+    </row>
+    <row r="530" spans="1:17" s="7" customFormat="1">
       <c r="A530" s="13"/>
       <c r="C530" s="12"/>
       <c r="G530" s="6"/>
-      <c r="R530" s="16"/>
-    </row>
-    <row r="531" spans="1:18" s="7" customFormat="1">
+      <c r="Q530" s="16"/>
+    </row>
+    <row r="531" spans="1:17" s="7" customFormat="1">
       <c r="A531" s="13"/>
       <c r="C531" s="12"/>
       <c r="G531" s="6"/>
-      <c r="R531" s="16"/>
-    </row>
-    <row r="532" spans="1:18" s="7" customFormat="1">
+      <c r="Q531" s="16"/>
+    </row>
+    <row r="532" spans="1:17" s="7" customFormat="1">
       <c r="A532" s="13"/>
       <c r="C532" s="12"/>
       <c r="G532" s="6"/>
-      <c r="R532" s="16"/>
-    </row>
-    <row r="533" spans="1:18" s="7" customFormat="1">
+      <c r="Q532" s="16"/>
+    </row>
+    <row r="533" spans="1:17" s="7" customFormat="1">
       <c r="A533" s="13"/>
       <c r="C533" s="12"/>
       <c r="G533" s="6"/>
-      <c r="R533" s="16"/>
-    </row>
-    <row r="534" spans="1:18" s="7" customFormat="1">
+      <c r="Q533" s="16"/>
+    </row>
+    <row r="534" spans="1:17" s="7" customFormat="1">
       <c r="A534" s="13"/>
       <c r="C534" s="12"/>
       <c r="G534" s="6"/>
-      <c r="R534" s="16"/>
-    </row>
-    <row r="535" spans="1:18" s="7" customFormat="1">
+      <c r="Q534" s="16"/>
+    </row>
+    <row r="535" spans="1:17" s="7" customFormat="1">
       <c r="A535" s="13"/>
       <c r="C535" s="12"/>
       <c r="G535" s="6"/>
-      <c r="R535" s="16"/>
-    </row>
-    <row r="536" spans="1:18" s="7" customFormat="1">
+      <c r="Q535" s="16"/>
+    </row>
+    <row r="536" spans="1:17" s="7" customFormat="1">
       <c r="A536" s="13"/>
       <c r="C536" s="12"/>
       <c r="G536" s="6"/>
-      <c r="R536" s="16"/>
-    </row>
-    <row r="537" spans="1:18" s="7" customFormat="1">
+      <c r="Q536" s="16"/>
+    </row>
+    <row r="537" spans="1:17" s="7" customFormat="1">
       <c r="A537" s="13"/>
       <c r="C537" s="12"/>
       <c r="G537" s="6"/>
-      <c r="R537" s="16"/>
-    </row>
-    <row r="538" spans="1:18" s="7" customFormat="1">
+      <c r="Q537" s="16"/>
+    </row>
+    <row r="538" spans="1:17" s="7" customFormat="1">
       <c r="A538" s="13"/>
       <c r="C538" s="12"/>
       <c r="G538" s="6"/>
-      <c r="R538" s="16"/>
-    </row>
-    <row r="539" spans="1:18" s="7" customFormat="1">
+      <c r="Q538" s="16"/>
+    </row>
+    <row r="539" spans="1:17" s="7" customFormat="1">
       <c r="A539" s="13"/>
       <c r="C539" s="12"/>
       <c r="G539" s="6"/>
-      <c r="R539" s="16"/>
-    </row>
-    <row r="540" spans="1:18" s="7" customFormat="1">
+      <c r="Q539" s="16"/>
+    </row>
+    <row r="540" spans="1:17" s="7" customFormat="1">
       <c r="A540" s="13"/>
       <c r="C540" s="12"/>
       <c r="G540" s="6"/>
-      <c r="R540" s="16"/>
-    </row>
-    <row r="541" spans="1:18" s="7" customFormat="1">
+      <c r="Q540" s="16"/>
+    </row>
+    <row r="541" spans="1:17" s="7" customFormat="1">
       <c r="A541" s="13"/>
       <c r="C541" s="12"/>
       <c r="G541" s="6"/>
-      <c r="R541" s="16"/>
-    </row>
-    <row r="542" spans="1:18" s="7" customFormat="1">
+      <c r="Q541" s="16"/>
+    </row>
+    <row r="542" spans="1:17" s="7" customFormat="1">
       <c r="A542" s="13"/>
       <c r="C542" s="12"/>
       <c r="G542" s="6"/>
-      <c r="R542" s="16"/>
-    </row>
-    <row r="543" spans="1:18" s="7" customFormat="1">
+      <c r="Q542" s="16"/>
+    </row>
+    <row r="543" spans="1:17" s="7" customFormat="1">
       <c r="A543" s="13"/>
       <c r="C543" s="12"/>
       <c r="G543" s="6"/>
-      <c r="R543" s="16"/>
-    </row>
-    <row r="544" spans="1:18" s="7" customFormat="1">
+      <c r="Q543" s="16"/>
+    </row>
+    <row r="544" spans="1:17" s="7" customFormat="1">
       <c r="A544" s="13"/>
       <c r="C544" s="12"/>
       <c r="G544" s="6"/>
-      <c r="R544" s="16"/>
-    </row>
-    <row r="545" spans="1:18" s="7" customFormat="1">
+      <c r="Q544" s="16"/>
+    </row>
+    <row r="545" spans="1:17" s="7" customFormat="1">
       <c r="A545" s="13"/>
       <c r="C545" s="12"/>
       <c r="G545" s="6"/>
-      <c r="R545" s="16"/>
-    </row>
-    <row r="546" spans="1:18" s="7" customFormat="1">
+      <c r="Q545" s="16"/>
+    </row>
+    <row r="546" spans="1:17" s="7" customFormat="1">
       <c r="A546" s="13"/>
       <c r="C546" s="12"/>
       <c r="G546" s="6"/>
-      <c r="R546" s="16"/>
-    </row>
-    <row r="547" spans="1:18" s="7" customFormat="1">
+      <c r="Q546" s="16"/>
+    </row>
+    <row r="547" spans="1:17" s="7" customFormat="1">
       <c r="A547" s="13"/>
       <c r="C547" s="12"/>
       <c r="G547" s="6"/>
-      <c r="R547" s="16"/>
-    </row>
-    <row r="548" spans="1:18" s="7" customFormat="1">
+      <c r="Q547" s="16"/>
+    </row>
+    <row r="548" spans="1:17" s="7" customFormat="1">
       <c r="A548" s="13"/>
       <c r="C548" s="12"/>
       <c r="G548" s="6"/>
-      <c r="R548" s="16"/>
-    </row>
-    <row r="549" spans="1:18" s="7" customFormat="1">
+      <c r="Q548" s="16"/>
+    </row>
+    <row r="549" spans="1:17" s="7" customFormat="1">
       <c r="A549" s="13"/>
       <c r="C549" s="12"/>
       <c r="G549" s="6"/>
-      <c r="R549" s="16"/>
-    </row>
-    <row r="550" spans="1:18" s="7" customFormat="1">
+      <c r="Q549" s="16"/>
+    </row>
+    <row r="550" spans="1:17" s="7" customFormat="1">
       <c r="A550" s="13"/>
       <c r="C550" s="12"/>
       <c r="G550" s="6"/>
-      <c r="R550" s="16"/>
-    </row>
-    <row r="551" spans="1:18" s="7" customFormat="1">
+      <c r="Q550" s="16"/>
+    </row>
+    <row r="551" spans="1:17" s="7" customFormat="1">
       <c r="A551" s="13"/>
       <c r="C551" s="12"/>
       <c r="G551" s="6"/>
-      <c r="R551" s="16"/>
-    </row>
-    <row r="552" spans="1:18" s="7" customFormat="1">
+      <c r="Q551" s="16"/>
+    </row>
+    <row r="552" spans="1:17" s="7" customFormat="1">
       <c r="A552" s="13"/>
       <c r="C552" s="12"/>
       <c r="G552" s="6"/>
-      <c r="R552" s="16"/>
-    </row>
-    <row r="553" spans="1:18" s="7" customFormat="1">
+      <c r="Q552" s="16"/>
+    </row>
+    <row r="553" spans="1:17" s="7" customFormat="1">
       <c r="A553" s="13"/>
       <c r="C553" s="12"/>
       <c r="G553" s="6"/>
-      <c r="R553" s="16"/>
-    </row>
-    <row r="554" spans="1:18" s="7" customFormat="1">
+      <c r="Q553" s="16"/>
+    </row>
+    <row r="554" spans="1:17" s="7" customFormat="1">
       <c r="A554" s="13"/>
       <c r="C554" s="12"/>
       <c r="G554" s="6"/>
-      <c r="R554" s="16"/>
-    </row>
-    <row r="555" spans="1:18" s="7" customFormat="1">
+      <c r="Q554" s="16"/>
+    </row>
+    <row r="555" spans="1:17" s="7" customFormat="1">
       <c r="A555" s="13"/>
       <c r="C555" s="12"/>
       <c r="G555" s="6"/>
-      <c r="R555" s="16"/>
-    </row>
-    <row r="556" spans="1:18" s="7" customFormat="1">
+      <c r="Q555" s="16"/>
+    </row>
+    <row r="556" spans="1:17" s="7" customFormat="1">
       <c r="A556" s="13"/>
       <c r="C556" s="12"/>
       <c r="G556" s="6"/>
-      <c r="R556" s="16"/>
-    </row>
-    <row r="557" spans="1:18" s="7" customFormat="1">
+      <c r="Q556" s="16"/>
+    </row>
+    <row r="557" spans="1:17" s="7" customFormat="1">
       <c r="A557" s="13"/>
       <c r="C557" s="12"/>
       <c r="G557" s="6"/>
-      <c r="R557" s="16"/>
-    </row>
-    <row r="558" spans="1:18" s="7" customFormat="1">
+      <c r="Q557" s="16"/>
+    </row>
+    <row r="558" spans="1:17" s="7" customFormat="1">
       <c r="A558" s="13"/>
       <c r="C558" s="12"/>
       <c r="G558" s="6"/>
-      <c r="R558" s="16"/>
-    </row>
-    <row r="559" spans="1:18" s="7" customFormat="1">
+      <c r="Q558" s="16"/>
+    </row>
+    <row r="559" spans="1:17" s="7" customFormat="1">
       <c r="A559" s="13"/>
       <c r="C559" s="12"/>
       <c r="G559" s="6"/>
-      <c r="R559" s="16"/>
-    </row>
-    <row r="560" spans="1:18" s="7" customFormat="1">
+      <c r="Q559" s="16"/>
+    </row>
+    <row r="560" spans="1:17" s="7" customFormat="1">
       <c r="A560" s="13"/>
       <c r="C560" s="12"/>
       <c r="G560" s="6"/>
-      <c r="R560" s="16"/>
-    </row>
-    <row r="561" spans="1:18" s="7" customFormat="1">
+      <c r="Q560" s="16"/>
+    </row>
+    <row r="561" spans="1:17" s="7" customFormat="1">
       <c r="A561" s="13"/>
       <c r="C561" s="12"/>
       <c r="G561" s="6"/>
-      <c r="R561" s="16"/>
-    </row>
-    <row r="562" spans="1:18" s="7" customFormat="1">
+      <c r="Q561" s="16"/>
+    </row>
+    <row r="562" spans="1:17" s="7" customFormat="1">
       <c r="A562" s="13"/>
       <c r="C562" s="12"/>
       <c r="G562" s="6"/>
-      <c r="R562" s="16"/>
-    </row>
-    <row r="563" spans="1:18" s="7" customFormat="1">
+      <c r="Q562" s="16"/>
+    </row>
+    <row r="563" spans="1:17" s="7" customFormat="1">
       <c r="A563" s="13"/>
       <c r="C563" s="12"/>
       <c r="G563" s="6"/>
-      <c r="R563" s="16"/>
-    </row>
-    <row r="564" spans="1:18" s="7" customFormat="1">
+      <c r="Q563" s="16"/>
+    </row>
+    <row r="564" spans="1:17" s="7" customFormat="1">
       <c r="A564" s="13"/>
       <c r="C564" s="12"/>
       <c r="G564" s="6"/>
-      <c r="R564" s="16"/>
-    </row>
-    <row r="565" spans="1:18" s="7" customFormat="1">
+      <c r="Q564" s="16"/>
+    </row>
+    <row r="565" spans="1:17" s="7" customFormat="1">
       <c r="A565" s="13"/>
       <c r="C565" s="12"/>
       <c r="G565" s="6"/>
-      <c r="R565" s="16"/>
-    </row>
-    <row r="566" spans="1:18" s="7" customFormat="1">
+      <c r="Q565" s="16"/>
+    </row>
+    <row r="566" spans="1:17" s="7" customFormat="1">
       <c r="A566" s="13"/>
       <c r="C566" s="12"/>
       <c r="G566" s="6"/>
-      <c r="R566" s="16"/>
-    </row>
-    <row r="567" spans="1:18" s="7" customFormat="1">
+      <c r="Q566" s="16"/>
+    </row>
+    <row r="567" spans="1:17" s="7" customFormat="1">
       <c r="A567" s="13"/>
       <c r="C567" s="12"/>
       <c r="G567" s="6"/>
-      <c r="R567" s="16"/>
-    </row>
-    <row r="568" spans="1:18" s="7" customFormat="1">
+      <c r="Q567" s="16"/>
+    </row>
+    <row r="568" spans="1:17" s="7" customFormat="1">
       <c r="A568" s="13"/>
       <c r="C568" s="12"/>
       <c r="G568" s="6"/>
-      <c r="R568" s="16"/>
-    </row>
-    <row r="569" spans="1:18" s="7" customFormat="1">
+      <c r="Q568" s="16"/>
+    </row>
+    <row r="569" spans="1:17" s="7" customFormat="1">
       <c r="A569" s="13"/>
       <c r="C569" s="12"/>
       <c r="G569" s="6"/>
-      <c r="R569" s="16"/>
-    </row>
-    <row r="570" spans="1:18" s="7" customFormat="1">
+      <c r="Q569" s="16"/>
+    </row>
+    <row r="570" spans="1:17" s="7" customFormat="1">
       <c r="A570" s="13"/>
       <c r="C570" s="12"/>
       <c r="G570" s="6"/>
-      <c r="R570" s="16"/>
-    </row>
-    <row r="571" spans="1:18" s="7" customFormat="1">
+      <c r="Q570" s="16"/>
+    </row>
+    <row r="571" spans="1:17" s="7" customFormat="1">
       <c r="A571" s="13"/>
       <c r="C571" s="12"/>
       <c r="G571" s="6"/>
-      <c r="R571" s="16"/>
-    </row>
-    <row r="572" spans="1:18" s="7" customFormat="1">
+      <c r="Q571" s="16"/>
+    </row>
+    <row r="572" spans="1:17" s="7" customFormat="1">
       <c r="A572" s="13"/>
       <c r="C572" s="12"/>
       <c r="G572" s="6"/>
-      <c r="R572" s="16"/>
-    </row>
-    <row r="573" spans="1:18" s="7" customFormat="1">
+      <c r="Q572" s="16"/>
+    </row>
+    <row r="573" spans="1:17" s="7" customFormat="1">
       <c r="A573" s="13"/>
       <c r="C573" s="12"/>
       <c r="G573" s="6"/>
-      <c r="R573" s="16"/>
-    </row>
-    <row r="574" spans="1:18" s="7" customFormat="1">
+      <c r="Q573" s="16"/>
+    </row>
+    <row r="574" spans="1:17" s="7" customFormat="1">
       <c r="A574" s="13"/>
       <c r="C574" s="12"/>
       <c r="G574" s="6"/>
-      <c r="R574" s="16"/>
-    </row>
-    <row r="575" spans="1:18" s="7" customFormat="1">
+      <c r="Q574" s="16"/>
+    </row>
+    <row r="575" spans="1:17" s="7" customFormat="1">
       <c r="A575" s="13"/>
       <c r="C575" s="12"/>
       <c r="G575" s="6"/>
-      <c r="R575" s="16"/>
-    </row>
-    <row r="576" spans="1:18" s="7" customFormat="1">
+      <c r="Q575" s="16"/>
+    </row>
+    <row r="576" spans="1:17" s="7" customFormat="1">
       <c r="A576" s="13"/>
       <c r="C576" s="12"/>
       <c r="G576" s="6"/>
-      <c r="R576" s="16"/>
-    </row>
-    <row r="577" spans="1:18" s="7" customFormat="1">
+      <c r="Q576" s="16"/>
+    </row>
+    <row r="577" spans="1:17" s="7" customFormat="1">
       <c r="A577" s="13"/>
       <c r="C577" s="12"/>
       <c r="G577" s="6"/>
-      <c r="R577" s="16"/>
-    </row>
-    <row r="578" spans="1:18" s="7" customFormat="1">
+      <c r="Q577" s="16"/>
+    </row>
+    <row r="578" spans="1:17" s="7" customFormat="1">
       <c r="A578" s="13"/>
       <c r="C578" s="12"/>
       <c r="G578" s="6"/>
-      <c r="R578" s="16"/>
-    </row>
-    <row r="579" spans="1:18" s="7" customFormat="1">
+      <c r="Q578" s="16"/>
+    </row>
+    <row r="579" spans="1:17" s="7" customFormat="1">
       <c r="A579" s="13"/>
       <c r="C579" s="12"/>
       <c r="G579" s="6"/>
-      <c r="R579" s="16"/>
-    </row>
-    <row r="580" spans="1:18" s="7" customFormat="1">
+      <c r="Q579" s="16"/>
+    </row>
+    <row r="580" spans="1:17" s="7" customFormat="1">
       <c r="A580" s="13"/>
       <c r="C580" s="12"/>
       <c r="G580" s="6"/>
-      <c r="R580" s="16"/>
-    </row>
-    <row r="581" spans="1:18" s="7" customFormat="1">
+      <c r="Q580" s="16"/>
+    </row>
+    <row r="581" spans="1:17" s="7" customFormat="1">
       <c r="A581" s="13"/>
       <c r="C581" s="12"/>
       <c r="G581" s="6"/>
-      <c r="R581" s="16"/>
-    </row>
-    <row r="582" spans="1:18" s="7" customFormat="1">
+      <c r="Q581" s="16"/>
+    </row>
+    <row r="582" spans="1:17" s="7" customFormat="1">
       <c r="A582" s="13"/>
       <c r="C582" s="12"/>
       <c r="G582" s="6"/>
-      <c r="R582" s="16"/>
-    </row>
-    <row r="583" spans="1:18" s="7" customFormat="1">
+      <c r="Q582" s="16"/>
+    </row>
+    <row r="583" spans="1:17" s="7" customFormat="1">
       <c r="A583" s="13"/>
       <c r="C583" s="12"/>
       <c r="G583" s="6"/>
-      <c r="R583" s="16"/>
-    </row>
-    <row r="584" spans="1:18" s="7" customFormat="1">
+      <c r="Q583" s="16"/>
+    </row>
+    <row r="584" spans="1:17" s="7" customFormat="1">
       <c r="A584" s="13"/>
       <c r="C584" s="12"/>
       <c r="G584" s="6"/>
-      <c r="R584" s="16"/>
-    </row>
-    <row r="585" spans="1:18" s="7" customFormat="1">
+      <c r="Q584" s="16"/>
+    </row>
+    <row r="585" spans="1:17" s="7" customFormat="1">
       <c r="A585" s="13"/>
       <c r="C585" s="12"/>
       <c r="G585" s="6"/>
-      <c r="R585" s="16"/>
-    </row>
-    <row r="586" spans="1:18" s="7" customFormat="1">
+      <c r="Q585" s="16"/>
+    </row>
+    <row r="586" spans="1:17" s="7" customFormat="1">
       <c r="A586" s="13"/>
       <c r="C586" s="12"/>
       <c r="G586" s="6"/>
-      <c r="R586" s="16"/>
-    </row>
-    <row r="587" spans="1:18" s="7" customFormat="1">
+      <c r="Q586" s="16"/>
+    </row>
+    <row r="587" spans="1:17" s="7" customFormat="1">
       <c r="A587" s="13"/>
       <c r="C587" s="12"/>
       <c r="G587" s="6"/>
-      <c r="R587" s="16"/>
-    </row>
-    <row r="588" spans="1:18" s="7" customFormat="1">
+      <c r="Q587" s="16"/>
+    </row>
+    <row r="588" spans="1:17" s="7" customFormat="1">
       <c r="A588" s="13"/>
       <c r="C588" s="12"/>
       <c r="G588" s="6"/>
-      <c r="R588" s="16"/>
-    </row>
-    <row r="589" spans="1:18" s="7" customFormat="1">
+      <c r="Q588" s="16"/>
+    </row>
+    <row r="589" spans="1:17" s="7" customFormat="1">
       <c r="A589" s="13"/>
       <c r="C589" s="12"/>
       <c r="G589" s="6"/>
-      <c r="R589" s="16"/>
-    </row>
-    <row r="590" spans="1:18" s="7" customFormat="1">
+      <c r="Q589" s="16"/>
+    </row>
+    <row r="590" spans="1:17" s="7" customFormat="1">
       <c r="A590" s="13"/>
       <c r="C590" s="12"/>
       <c r="G590" s="6"/>
-      <c r="R590" s="16"/>
-    </row>
-    <row r="591" spans="1:18" s="7" customFormat="1">
+      <c r="Q590" s="16"/>
+    </row>
+    <row r="591" spans="1:17" s="7" customFormat="1">
       <c r="A591" s="13"/>
       <c r="C591" s="12"/>
       <c r="G591" s="6"/>
-      <c r="R591" s="16"/>
-    </row>
-    <row r="592" spans="1:18" s="7" customFormat="1">
+      <c r="Q591" s="16"/>
+    </row>
+    <row r="592" spans="1:17" s="7" customFormat="1">
       <c r="A592" s="13"/>
       <c r="C592" s="12"/>
       <c r="G592" s="6"/>
-      <c r="R592" s="16"/>
-    </row>
-    <row r="593" spans="1:18" s="7" customFormat="1">
+      <c r="Q592" s="16"/>
+    </row>
+    <row r="593" spans="1:17" s="7" customFormat="1">
       <c r="A593" s="13"/>
       <c r="C593" s="12"/>
       <c r="G593" s="6"/>
-      <c r="R593" s="16"/>
-    </row>
-    <row r="594" spans="1:18" s="7" customFormat="1">
+      <c r="Q593" s="16"/>
+    </row>
+    <row r="594" spans="1:17" s="7" customFormat="1">
       <c r="A594" s="13"/>
       <c r="C594" s="12"/>
       <c r="G594" s="6"/>
-      <c r="R594" s="16"/>
-    </row>
-    <row r="595" spans="1:18" s="7" customFormat="1">
+      <c r="Q594" s="16"/>
+    </row>
+    <row r="595" spans="1:17" s="7" customFormat="1">
       <c r="A595" s="13"/>
       <c r="C595" s="12"/>
       <c r="G595" s="6"/>
-      <c r="R595" s="16"/>
-    </row>
-    <row r="596" spans="1:18" s="7" customFormat="1">
+      <c r="Q595" s="16"/>
+    </row>
+    <row r="596" spans="1:17" s="7" customFormat="1">
       <c r="A596" s="13"/>
       <c r="C596" s="12"/>
       <c r="G596" s="6"/>
-      <c r="R596" s="16"/>
+      <c r="Q596" s="16"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:R596">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:Q596">
     <sortCondition ref="B2:B596"/>
   </sortState>
   <hyperlinks>

</xml_diff>